<commit_message>
code + files modifications
</commit_message>
<xml_diff>
--- a/documents/ParaBank_RTM.xlsx
+++ b/documents/ParaBank_RTM.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="93">
   <si>
     <t xml:space="preserve">Req ID</t>
   </si>
@@ -273,6 +273,18 @@
   </si>
   <si>
     <t xml:space="preserve">TC-PSF-01 to TC-PSF-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REQ-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New customers must be able to register for an account by submitting valid, unique personal and credential data; the system must reject invalid or incomplete submissions and enforce unique usernames and matching passwords.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Registration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-REG-01 to TC-REG-19</t>
   </si>
   <si>
     <t xml:space="preserve">Metric</t>
@@ -415,8 +427,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -432,15 +448,19 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -733,452 +753,475 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="16"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G2" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="G2" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G3" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="G3" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G4" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="G4" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="G5" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="G5" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="G6" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+      <c r="G6" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="G7" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="G7" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="G8" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+      <c r="G8" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F9" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="G9" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="G9" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="G10" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+      <c r="G10" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="E11" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="F11" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="G11" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+      <c r="G11" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E12" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="F12" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="G12" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
+      <c r="G12" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D13" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="E13" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="F13" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="G13" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+      <c r="G13" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="E14" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="F14" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G14" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
+      <c r="G14" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D15" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="E15" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="F15" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G15" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
+      <c r="G15" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="D16" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="E16" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="F16" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="G16" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="s">
+      <c r="G16" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="D17" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="E17" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="F17" s="2" t="s">
+      <c r="F17" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="G17" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
+      <c r="G17" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="D18" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="E18" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="F18" s="2" t="s">
+      <c r="F18" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="G18" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
+      <c r="G18" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C19" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="D19" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="E19" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="F19" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="G19" s="3" t="s">
+      <c r="G19" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G20" s="5" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1203,55 +1246,55 @@
   <dimension ref="A1:B6"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="B2" s="5" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" s="5" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="B4" s="5" t="n">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="B2" s="7" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="7" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="B4" s="7" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="B5" s="5" t="n">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="B5" s="7" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="B6" s="6" t="n">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B6" s="8" t="n">
         <f aca="false">B3/B2</f>
         <v>1</v>
       </c>

</xml_diff>